<commit_message>
Rev C: use turnkey PTH USB-C and Standard DRC clearances
</commit_message>
<xml_diff>
--- a/MACROFAB-UPLOADS/02-swansong-usb-bom.xlsx
+++ b/MACROFAB-UPLOADS/02-swansong-usb-bom.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="Rd10c5a541b71439b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="R0ee0610e476a44b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -379,7 +379,7 @@
         <x:v>J1</x:v>
       </x:c>
       <x:c r="B3" s="11" t="str">
-        <x:v>USB4110-GF-A</x:v>
+        <x:v>USB4085-GF-A</x:v>
       </x:c>
       <x:c r="C3" s="11" t="str">
         <x:v>GCT</x:v>
@@ -388,7 +388,7 @@
         <x:v>USB-C 2.0 receptacle</x:v>
       </x:c>
       <x:c r="E3" s="11" t="str">
-        <x:v>GCT USB4110</x:v>
+        <x:v>GCT USB4085 PTH</x:v>
       </x:c>
       <x:c r="F3" s="12" t="n">
         <x:v>1</x:v>

</xml_diff>